<commit_message>
Added Query to get Variance by zone.
</commit_message>
<xml_diff>
--- a/data/shift_data.xlsx
+++ b/data/shift_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\somto\OneDrive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CEC62A0-2F6E-40FC-B3CE-8C0B6F6E03D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC23B7E-AAB1-4979-8D36-90517629817F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D9275F6-8CE3-4795-A668-2BEF9AD47A96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8D9275F6-8CE3-4795-A668-2BEF9AD47A96}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
   <si>
     <t>Date</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>Zone C</t>
+  </si>
+  <si>
+    <t>Actual_Tonnes</t>
   </si>
 </sst>
 </file>
@@ -504,7 +507,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>